<commit_message>
Refonte graphique, nouvel algorithme
</commit_message>
<xml_diff>
--- a/instructs.xlsx
+++ b/instructs.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\p00688\Documents\PsychoPy\IAT_SENSE\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\p00688\Documents\PsychoPy\IAT 2.0\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{027CFD7F-176F-44CD-8928-A48E1B54626C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{742D8C81-9126-43C2-BE7E-E7FC91448B4F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="10690" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -30,15 +30,15 @@
     <t>instruct_text</t>
   </si>
   <si>
-    <t>Des mots vont apparaître au centre de l'écran. Vous devrez les classer en utilisant les touches "E" et "I" de votre clavier.
-Essayez d'être le plus rapide possible et de ne pas faire d'erreurs.</t>
-  </si>
-  <si>
     <t>pageNum</t>
   </si>
   <si>
-    <t>Les touches "E" et "I" du clavier seront toujours associées à une catégorie qui sera affichée.
-Chaque mot a une classification correcte. En cas d'erreur, elle sera affichée et vous devrez appuyer sur la touche correcte pour continuer.
+    <t>Des mots vous seront présentés un par un au centre de l’écran. 
+Vous devrez les classer aussi vite que possible sans faire d’erreurs dans la ou les catégories situées en haut à gauche et à droite de l’écran.
+Les touches "E" et "I" seront associées à une catégorie et vous permettront de répondre.</t>
+  </si>
+  <si>
+    <t>Chaque mot a une classification correcte. En cas d'erreur, vous devez appuyer sur la touche correcte pour continuer.
 Le test ne donne pas de résultat si vous répondez trop rapidement ou trop lentement.
 Appuyez sur la barre espace pour passer à l'étape suivante.</t>
   </si>
@@ -375,7 +375,7 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B1" t="s">
         <v>0</v>
@@ -386,10 +386,10 @@
         <v>1</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="75" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" ht="60" x14ac:dyDescent="0.25">
       <c r="A3" s="2">
         <v>2</v>
       </c>

</xml_diff>